<commit_message>
Add USD rows under KVB CNY gateways and flag missed fees.
KVB Generate D&W now passes --usd-shadow, --fee-currency-suffix, --warn-high-pct, and --cny-rate-check. A DPM run without those flags keeps the previous workbook.

Co-authored-by: Bayu Darmawan <gorillaworkout@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Template KVB Plus.xlsx
+++ b/Template KVB Plus.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xero" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handling Fee" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Transfer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="D" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="W" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Xero" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Handling Fee" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Transfer'!$A$2:$S$2</definedName>
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,10 +70,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -144,6 +152,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Template KVB Plus</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Rate guide: +8 = flat 8 per transaction (the plus sign is required). 1.5%+50 = 1.5% of the transaction plus a flat 50. 0.45%,min 90 = 0.45%, but at least 90. A plain number 8 is read as 800%, not as a flat fee. Write +8 for a flat fee.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Rate guide: +8 = flat 8 per transaction (the plus sign is required). 1.5%+50 = 1.5% of the transaction plus a flat 50. 0.45%,min 90 = 0.45%, but at least 90. A plain number 8 is read as 800%, not as a flat fee. Write +8 for a flat fee.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -465,25 +493,11 @@
           <t>汇出</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>收款</t>
         </is>
       </c>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
@@ -1102,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1110,9 +1124,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="88" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Payment Channel</t>
@@ -1136,11 +1151,17 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Remark</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Rate guide: +8 = flat 8 per transaction (the plus sign is required). 1.5%+50 = 1.5% of the transaction plus a flat 50. 0.45%,min 90 = 0.45%, but at least 90. A plain number 8 is read as 800%, not as a flat fee. Write +8 for a flat fee.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add USD rows under KVB CNY gateways and flag missed fees. (#9)
KVB Generate D&W now passes --usd-shadow, --fee-currency-suffix, --warn-high-pct, and --cny-rate-check. A DPM run without those flags keeps the previous workbook.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Bayu Darmawan <gorillaworkout@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Template KVB Plus.xlsx
+++ b/Template KVB Plus.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transfer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="W" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Xero" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handling Fee" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Transfer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="D" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="W" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Xero" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Handling Fee" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Transfer'!$A$2:$S$2</definedName>
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,11 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,10 +70,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -144,6 +152,26 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Template KVB Plus</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Rate guide: +8 = flat 8 per transaction (the plus sign is required). 1.5%+50 = 1.5% of the transaction plus a flat 50. 0.45%,min 90 = 0.45%, but at least 90. A plain number 8 is read as 800%, not as a flat fee. Write +8 for a flat fee.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Rate guide: +8 = flat 8 per transaction (the plus sign is required). 1.5%+50 = 1.5% of the transaction plus a flat 50. 0.45%,min 90 = 0.45%, but at least 90. A plain number 8 is read as 800%, not as a flat fee. Write +8 for a flat fee.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -465,25 +493,11 @@
           <t>汇出</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="inlineStr">
         <is>
           <t>收款</t>
         </is>
       </c>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
       <c r="Q1" s="1" t="n"/>
       <c r="R1" s="1" t="n"/>
       <c r="S1" s="1" t="n"/>
@@ -1102,7 +1116,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1110,9 +1124,10 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="88" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Payment Channel</t>
@@ -1136,11 +1151,17 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Remark</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Rate guide: +8 = flat 8 per transaction (the plus sign is required). 1.5%+50 = 1.5% of the transaction plus a flat 50. 0.45%,min 90 = 0.45%, but at least 90. A plain number 8 is read as 800%, not as a flat fee. Write +8 for a flat fee.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>